<commit_message>
Lecturer dedup, merged course segregation, level 200+ early slot constraint, fixes
- Normalize lecturer names via LECTURER_ALIASES in GET /api/lecturers and collapse
- Clean up lecturers.xlsx (74 canonical names) and courses.xlsx (319 values)
- Separate E. Arhinful from Dr D. Arhinful as distinct lecturers
- Merge R. K. Amoah into Dr R. K. Amoah
- Segregate merged co-taught courses as independent rows (individual code/name/group_id)
- Fix KeyError on 'section' in solve summary (use .get() for safe access)
- Add level 200+ in-person sessions cannot start before 08:30 constraint
- UI: simplify courses page (TPC button), add course at top with auto-scroll
- Excel: multi-row ONLINE/FIELD WORK sheets, single-cell merge guard
</commit_message>
<xml_diff>
--- a/data/lecturers.xlsx
+++ b/data/lecturers.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A142"/>
+  <dimension ref="A1:A75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,980 +433,511 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ADJARDJA</t>
+          <t>ADOMAKO-ANSAH</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ADOMAKO-ANSAH</t>
+          <t>Ako Hayford</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ADU KYEREMH</t>
+          <t>Akorli</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ADU-GYEMFI</t>
+          <t>Assoc Prof J. Acquah</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ADZAKOR</t>
+          <t>Assoc Prof Ziggeh</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AKO HAYFORD</t>
+          <t>Attafuah</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AKORLI</t>
+          <t>Dr A. A. Amponsah</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AKYEN</t>
+          <t>Dr A. Asante-Annor</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AMPOFI</t>
+          <t>Dr A. K. Kwansah Ansah</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AMPOMAH</t>
+          <t>Dr Adu-Gyemfi</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ANAFO</t>
+          <t>Dr Anafo</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ANNAN</t>
+          <t>Dr C. A. Komolafe</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ARHINFUL</t>
+          <t>Dr D. Arhinful</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ASHUN</t>
+          <t>Dr D. K. Tortor</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ASSOC PROF TAGOE</t>
+          <t>Dr E. A. Nti</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ASSOC PROF ZIGGAH</t>
+          <t>Dr E. Ashun</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ATTAFUAH</t>
+          <t>Dr E. K. Ampomah</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ATTATSI</t>
+          <t>Dr E. M. Martey</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Assoc Prof J. Acquah</t>
+          <t>Dr E. N. Asare</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>D. ARHINFUL</t>
+          <t>Dr E. Quansah</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DR A. ASANTE-ANNOR</t>
+          <t>Dr F. Annan</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DR A. ASARE-ANNOR</t>
+          <t>Dr F. Dartey</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DR A. K. KWANSAH ANSAH</t>
+          <t>Dr G. Owusu</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>DR ADU-GYEMFI</t>
+          <t>Dr Howard-Ferguson</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>DR AMOAH</t>
+          <t>Dr I. K. Attatsi</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DR ANAFO</t>
+          <t>Dr I. Ofori</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DR ASHUN</t>
+          <t>Dr J. Annan</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DR C. KOMOLAFE</t>
+          <t>Dr J. S. Ansah</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DR DARTEH</t>
+          <t>Dr J. Seidu</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>DR E. ASHUN</t>
+          <t>Dr Klu</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>DR E. K. AMPOMAH</t>
+          <t>Dr R. Annan</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>DR E. N. ASARE</t>
+          <t>Dr R. K. Amoah</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DR E. QUANSAH</t>
+          <t>Dr R. K. Kuffour</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DR F. ANNAN</t>
+          <t>Dr R. N. Nketsiah</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DR F. DARTEY</t>
+          <t>Dr S. Sebbeh-Newton</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>DR G OWUSU</t>
+          <t>Dr T. Kwantwi</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>DR G. OWUSU</t>
+          <t>Dr Yakah</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DR HOWARD-FERGUSON</t>
+          <t>E. Adu Kyeremeh</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>DR I. ATTATSI</t>
+          <t>E. Annan-Boah</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DR J SEIDU</t>
+          <t>E. Arhinful</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>DR J. ANNAN</t>
+          <t>E. Asante</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>DR J. S. ANSAH</t>
+          <t>E. Benyarku</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>DR KLU</t>
+          <t>E. Mensah</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>DR KWANSH ANSAH</t>
+          <t>E. N. Asare</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>DR M. POKU</t>
+          <t>E. Obu</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>DR N. NKETSIAH</t>
+          <t>Ewusi-Essoun</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>DR NTI</t>
+          <t>F. Mumuni</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>DR OFORI</t>
+          <t>F. Tabase</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>DR POKU</t>
+          <t>G. M. Tetteh</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>DR R. AMOAH</t>
+          <t>I. Ampofi</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>DR R. ANNAN</t>
+          <t>I. K. Prah</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>DR R. F. ANNAN</t>
+          <t>I. Kwofie</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>DR R. KUFFOUR</t>
+          <t>J. Ellis</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>DR R. NSIAH</t>
+          <t>M. B. Poku</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>DR SEBBEH-NEWTON</t>
+          <t>M. O. Alhassan</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>DR TORTOR</t>
+          <t>N. K. Adzakor</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>DR TOTROR</t>
+          <t>Owusu-Bempah</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>DR YAKAH</t>
+          <t>Prof A. Simons</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Dr A. A. Amponsah</t>
+          <t>Prof Affam</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Dr A. K. Kwansah Ansah</t>
+          <t>Prof I. Yakubu</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Dr D. Arhinful</t>
+          <t>Prof Lawal</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Dr E. K. Ampomah</t>
+          <t>Prof S. Nunoo</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Dr E. M. Martey</t>
+          <t>Prof Tagoe</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Dr G. Owusu</t>
+          <t>Prof W. Adjardjah</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Dr I. K. Attatsi</t>
+          <t>Prof Ziggeh</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Dr I. Ofori</t>
+          <t>Rev S. Odoom</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Dr J. Seidu</t>
+          <t>S. Alhassan</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Dr R. N. Nketsiah</t>
+          <t>S. K. Dankwah</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Dr S. Sebbeh-Newton</t>
+          <t>S. K. Yormesor</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Dr T. Kwantwi</t>
+          <t>S. L. Afful</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>E. ARHINFUL</t>
+          <t>S. Nanor</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>E. ARHIUNFUL</t>
+          <t>T. Akyen</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>E. Adu Kyeremeh</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>E. Annan-Boah</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>E. Asante</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>E. Benyarku</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>E. MENSAH</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>E. N. Asare</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>E. Obu</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>E. QUANSAH</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>Ewusi-Essoun</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>F. MUMUNI</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>F. Tabase</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>G OWUSU</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>G.M. TETTEH</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>HAWARD-FERGUSON</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>HAWARD-FURGUSON</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>HOWARD-FERGUSON</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>I. AMPOFI</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>I. K. Prah</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>I. Kwofie</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>J. ANSAH</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>J. Ellis</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>J. S. ANSAH</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>KOMOLAFE</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>KWANSAH ANSAH</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>M. B. Poku</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>M. O. ALHASSAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>M.O ALHASSAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>M.O. ALHASSAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>MENSAH</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>MUMUNI</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>NANOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>NKETSIA</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>NKETSIAH</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>NTI</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>ODOOM</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>Owusu-Bempah</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>PROF A. SIMONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>PROF ADJARDJA</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>PROF ADJARDJAH</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>PROF ADJARJAH</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>PROF AFFAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>PROF LAWAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>PROF NUNOO</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>PROF S. NUNOO</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>PROF TAGOE</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>PROF YAKUBU</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>R. K. Amoah</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>R. KUFFOUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>R. NSIAH</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>R. PROF YAKUBU</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>REV ODOOM</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>REV S.ODOOM</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>Rev S. Odoom</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>S. AFFUL</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>S. ALHASSAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>S. K. Dankwah</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>S. K. Yormesor</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>S. L. AFFUL</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>S. NANOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>SEIDU</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>T. AKYEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>TABASE</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>TAGOE</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>TORTOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>YAKAH</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>YAKUBU</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>YALLEY</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>ZIGGAH</t>
+          <t>Yalley</t>
         </is>
       </c>
     </row>

</xml_diff>